<commit_message>
Let answers count and summarise; explain not-found in whole-document mode
"Store visits per month" was answered "I couldn't find this" although
all six visit reports (all in August 2026) were sent to Claude: the
grounding rule told it to reply not-found whenever the excerpts didn't
contain the answer verbatim. The rule now allows counting, totalling,
grouping and summarising what the documents state, asks for partial
answers that say what's missing, and keeps not-found for when nothing is
relevant (still no outside knowledge). Whole-document not-found answers
now say how many documents Claude read. Added the question to the
evaluation pack as A9.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/local-qa/eval/Evaluation_Scoresheet.xlsx
+++ b/local-qa/eval/Evaluation_Scoresheet.xlsx
@@ -714,19 +714,19 @@
         </is>
       </c>
       <c r="B2" s="6">
-        <f>COUNTIF('Test cases'!$B$3:$B$20,"A: Unstructured")</f>
+        <f>COUNTIF('Test cases'!$B$3:$B$21,"A: Unstructured")</f>
         <v/>
       </c>
       <c r="C2" s="6">
-        <f>COUNTIF('Test cases'!$B$3:$B$20,"B: Sales")</f>
+        <f>COUNTIF('Test cases'!$B$3:$B$21,"B: Sales")</f>
         <v/>
       </c>
       <c r="D2" s="6">
-        <f>COUNTIF('Test cases'!$B$3:$B$20,"Cross-use-case")</f>
+        <f>COUNTIF('Test cases'!$B$3:$B$21,"Cross-use-case")</f>
         <v/>
       </c>
       <c r="E2" s="6">
-        <f>COUNTA('Test cases'!$A$3:$A$20)</f>
+        <f>COUNTA('Test cases'!$A$3:$A$21)</f>
         <v/>
       </c>
       <c r="F2" s="6" t="inlineStr"/>
@@ -738,19 +738,19 @@
         </is>
       </c>
       <c r="B3" s="6">
-        <f>COUNTIFS('Test cases'!$B$3:$B$20,"A: Unstructured",'Test cases'!$J$3:$J$20,"&lt;&gt;")</f>
+        <f>COUNTIFS('Test cases'!$B$3:$B$21,"A: Unstructured",'Test cases'!$J$3:$J$21,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="C3" s="6">
-        <f>COUNTIFS('Test cases'!$B$3:$B$20,"B: Sales",'Test cases'!$J$3:$J$20,"&lt;&gt;")</f>
+        <f>COUNTIFS('Test cases'!$B$3:$B$21,"B: Sales",'Test cases'!$J$3:$J$21,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="D3" s="6">
-        <f>COUNTIFS('Test cases'!$B$3:$B$20,"Cross-use-case",'Test cases'!$J$3:$J$20,"&lt;&gt;")</f>
+        <f>COUNTIFS('Test cases'!$B$3:$B$21,"Cross-use-case",'Test cases'!$J$3:$J$21,"&lt;&gt;")</f>
         <v/>
       </c>
       <c r="E3" s="6">
-        <f>COUNT('Test cases'!$J$3:$J$20)</f>
+        <f>COUNT('Test cases'!$J$3:$J$21)</f>
         <v/>
       </c>
       <c r="F3" s="6" t="inlineStr"/>
@@ -762,19 +762,19 @@
         </is>
       </c>
       <c r="B4" s="6">
-        <f>COUNTIFS('Test cases'!$B$3:$B$20,"A: Unstructured",'Test cases'!$J$3:$J$20,2)</f>
+        <f>COUNTIFS('Test cases'!$B$3:$B$21,"A: Unstructured",'Test cases'!$J$3:$J$21,2)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIFS('Test cases'!$B$3:$B$20,"B: Sales",'Test cases'!$J$3:$J$20,2)</f>
+        <f>COUNTIFS('Test cases'!$B$3:$B$21,"B: Sales",'Test cases'!$J$3:$J$21,2)</f>
         <v/>
       </c>
       <c r="D4" s="6">
-        <f>COUNTIFS('Test cases'!$B$3:$B$20,"Cross-use-case",'Test cases'!$J$3:$J$20,2)</f>
+        <f>COUNTIFS('Test cases'!$B$3:$B$21,"Cross-use-case",'Test cases'!$J$3:$J$21,2)</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>COUNTIF('Test cases'!$J$3:$J$20,2)</f>
+        <f>COUNTIF('Test cases'!$J$3:$J$21,2)</f>
         <v/>
       </c>
       <c r="F4" s="6" t="inlineStr"/>
@@ -786,19 +786,19 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>IFERROR(SUMIFS('Test cases'!$J$3:$J$20,'Test cases'!$B$3:$B$20,"A: Unstructured")/(2*COUNTIFS('Test cases'!$B$3:$B$20,"A: Unstructured",'Test cases'!$J$3:$J$20,"&lt;&gt;")),"")</f>
+        <f>IFERROR(SUMIFS('Test cases'!$J$3:$J$21,'Test cases'!$B$3:$B$21,"A: Unstructured")/(2*COUNTIFS('Test cases'!$B$3:$B$21,"A: Unstructured",'Test cases'!$J$3:$J$21,"&lt;&gt;")),"")</f>
         <v/>
       </c>
       <c r="C5" s="7">
-        <f>IFERROR(SUMIFS('Test cases'!$J$3:$J$20,'Test cases'!$B$3:$B$20,"B: Sales")/(2*COUNTIFS('Test cases'!$B$3:$B$20,"B: Sales",'Test cases'!$J$3:$J$20,"&lt;&gt;")),"")</f>
+        <f>IFERROR(SUMIFS('Test cases'!$J$3:$J$21,'Test cases'!$B$3:$B$21,"B: Sales")/(2*COUNTIFS('Test cases'!$B$3:$B$21,"B: Sales",'Test cases'!$J$3:$J$21,"&lt;&gt;")),"")</f>
         <v/>
       </c>
       <c r="D5" s="7">
-        <f>IFERROR(SUMIFS('Test cases'!$J$3:$J$20,'Test cases'!$B$3:$B$20,"Cross-use-case")/(2*COUNTIFS('Test cases'!$B$3:$B$20,"Cross-use-case",'Test cases'!$J$3:$J$20,"&lt;&gt;")),"")</f>
+        <f>IFERROR(SUMIFS('Test cases'!$J$3:$J$21,'Test cases'!$B$3:$B$21,"Cross-use-case")/(2*COUNTIFS('Test cases'!$B$3:$B$21,"Cross-use-case",'Test cases'!$J$3:$J$21,"&lt;&gt;")),"")</f>
         <v/>
       </c>
       <c r="E5" s="7">
-        <f>IFERROR(SUM('Test cases'!$J$3:$J$20)/(2*COUNT('Test cases'!$J$3:$J$20)),"")</f>
+        <f>IFERROR(SUM('Test cases'!$J$3:$J$21)/(2*COUNT('Test cases'!$J$3:$J$21)),"")</f>
         <v/>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -814,19 +814,19 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>IFERROR(COUNTIFS('Test cases'!$B$3:$B$20,"A: Unstructured",'Test cases'!$K$3:$K$20,"Y")/COUNTIFS('Test cases'!$B$3:$B$20,"A: Unstructured",'Test cases'!$K$3:$K$20,"?*"),"")</f>
+        <f>IFERROR(COUNTIFS('Test cases'!$B$3:$B$21,"A: Unstructured",'Test cases'!$K$3:$K$21,"Y")/COUNTIFS('Test cases'!$B$3:$B$21,"A: Unstructured",'Test cases'!$K$3:$K$21,"?*"),"")</f>
         <v/>
       </c>
       <c r="C6" s="7">
-        <f>IFERROR(COUNTIFS('Test cases'!$B$3:$B$20,"B: Sales",'Test cases'!$K$3:$K$20,"Y")/COUNTIFS('Test cases'!$B$3:$B$20,"B: Sales",'Test cases'!$K$3:$K$20,"?*"),"")</f>
+        <f>IFERROR(COUNTIFS('Test cases'!$B$3:$B$21,"B: Sales",'Test cases'!$K$3:$K$21,"Y")/COUNTIFS('Test cases'!$B$3:$B$21,"B: Sales",'Test cases'!$K$3:$K$21,"?*"),"")</f>
         <v/>
       </c>
       <c r="D6" s="7">
-        <f>IFERROR(COUNTIFS('Test cases'!$B$3:$B$20,"Cross-use-case",'Test cases'!$K$3:$K$20,"Y")/COUNTIFS('Test cases'!$B$3:$B$20,"Cross-use-case",'Test cases'!$K$3:$K$20,"?*"),"")</f>
+        <f>IFERROR(COUNTIFS('Test cases'!$B$3:$B$21,"Cross-use-case",'Test cases'!$K$3:$K$21,"Y")/COUNTIFS('Test cases'!$B$3:$B$21,"Cross-use-case",'Test cases'!$K$3:$K$21,"?*"),"")</f>
         <v/>
       </c>
       <c r="E6" s="7">
-        <f>IFERROR(COUNTIF('Test cases'!$K$3:$K$20,"Y")/COUNTIF('Test cases'!$K$3:$K$20,"?*"),"")</f>
+        <f>IFERROR(COUNTIF('Test cases'!$K$3:$K$21,"Y")/COUNTIF('Test cases'!$K$3:$K$21,"?*"),"")</f>
         <v/>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -842,19 +842,19 @@
         </is>
       </c>
       <c r="B7" s="6">
-        <f>COUNTIFS('Test cases'!$B$3:$B$20,"A: Unstructured",'Test cases'!$L$3:$L$20,"Y")</f>
+        <f>COUNTIFS('Test cases'!$B$3:$B$21,"A: Unstructured",'Test cases'!$L$3:$L$21,"Y")</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('Test cases'!$B$3:$B$20,"B: Sales",'Test cases'!$L$3:$L$20,"Y")</f>
+        <f>COUNTIFS('Test cases'!$B$3:$B$21,"B: Sales",'Test cases'!$L$3:$L$21,"Y")</f>
         <v/>
       </c>
       <c r="D7" s="6">
-        <f>COUNTIFS('Test cases'!$B$3:$B$20,"Cross-use-case",'Test cases'!$L$3:$L$20,"Y")</f>
+        <f>COUNTIFS('Test cases'!$B$3:$B$21,"Cross-use-case",'Test cases'!$L$3:$L$21,"Y")</f>
         <v/>
       </c>
       <c r="E7" s="6">
-        <f>COUNTIF('Test cases'!$L$3:$L$20,"Y")</f>
+        <f>COUNTIF('Test cases'!$L$3:$L$21,"Y")</f>
         <v/>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -870,19 +870,19 @@
         </is>
       </c>
       <c r="B8" s="8">
-        <f>IFERROR(AVERAGEIFS('Test cases'!$M$3:$M$20,'Test cases'!$B$3:$B$20,"A: Unstructured"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Test cases'!$M$3:$M$21,'Test cases'!$B$3:$B$21,"A: Unstructured"),"")</f>
         <v/>
       </c>
       <c r="C8" s="8">
-        <f>IFERROR(AVERAGEIFS('Test cases'!$M$3:$M$20,'Test cases'!$B$3:$B$20,"B: Sales"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Test cases'!$M$3:$M$21,'Test cases'!$B$3:$B$21,"B: Sales"),"")</f>
         <v/>
       </c>
       <c r="D8" s="8">
-        <f>IFERROR(AVERAGEIFS('Test cases'!$M$3:$M$20,'Test cases'!$B$3:$B$20,"Cross-use-case"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Test cases'!$M$3:$M$21,'Test cases'!$B$3:$B$21,"Cross-use-case"),"")</f>
         <v/>
       </c>
       <c r="E8" s="8">
-        <f>IFERROR(AVERAGE('Test cases'!$M$3:$M$20),"")</f>
+        <f>IFERROR(AVERAGE('Test cases'!$M$3:$M$21),"")</f>
         <v/>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -909,7 +909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1472,42 +1472,42 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>A9</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>B: Sales</t>
+          <t>A: Unstructured</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>Lookup</t>
+          <t>Derived count</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>What discount was given on the Ember Room Heater in April 2026, and why?</t>
+          <t>How many store visits were there per month?</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>25% clearance discount (April and May) to reduce winter stock; standard home comfort discount is 8%.</t>
+          <t>6 store visits, all in August 2026 (12, 14, 18, 20, 22 and 25 August); none in any other month.</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>25%, clearance reason.</t>
+          <t>6 visits, all August.</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>2 = both; 1 = number only; 0 = wrong.</t>
+          <t>2 = 6 in August and none elsewhere; 1 = August only or wrong count; 0 = 'not found' or invented months.</t>
         </is>
       </c>
       <c r="H11" s="12" t="inlineStr">
         <is>
-          <t>Default settings</t>
+          <t>Default settings (found in real testing: an over-strict prompt made the tool answer 'not found')</t>
         </is>
       </c>
       <c r="I11" s="13" t="n"/>
@@ -1520,7 +1520,7 @@
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
@@ -1530,27 +1530,27 @@
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Narrative</t>
+          <t>Lookup</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>Why did Drift Air Cooler sales peak in May?</t>
+          <t>What discount was given on the Ember Room Heater in April 2026, and why?</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>A heatwave across North and West India in May (commentary); sales eased from July with the monsoon.</t>
+          <t>25% clearance discount (April and May) to reduce winter stock; standard home comfort discount is 8%.</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>Heatwave, May.</t>
+          <t>25%, clearance reason.</t>
         </is>
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>2 = cause + timing; 1 = cause only; 0 = wrong.</t>
+          <t>2 = both; 1 = number only; 0 = wrong.</t>
         </is>
       </c>
       <c r="H12" s="12" t="inlineStr">
@@ -1568,7 +1568,7 @@
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
@@ -1578,27 +1578,27 @@
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>Chart (exact numbers)</t>
+          <t>Narrative</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Plot monthly units sold of Drift Air Cooler as a line chart.</t>
+          <t>Why did Drift Air Cooler sales peak in May?</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>Proposal table, then line chart with all regions summed: April 1,095; May 1,469; June 1,150; July 598; August 398; September 323.</t>
+          <t>A heatwave across North and West India in May (commentary); sales eased from July with the monsoon.</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Values match exactly; source shows Sales_FY27_H1.xlsx sheet Transactions.</t>
+          <t>Heatwave, May.</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>2 = exact values and plotted after confirm; 1 = right shape, wrong grouping; 0 = wrong numbers.</t>
+          <t>2 = cause + timing; 1 = cause only; 0 = wrong.</t>
         </is>
       </c>
       <c r="H13" s="12" t="inlineStr">
@@ -1616,7 +1616,7 @@
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B14" s="12" t="inlineStr">
@@ -1631,22 +1631,22 @@
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>Bar chart of total net revenue by product for H1.</t>
+          <t>Plot monthly units sold of Drift Air Cooler as a line chart.</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Bar chart, values (₹): Cascade Water Purifier ₹40,085,016; Drift Air Cooler ₹39,353,430; Breeze Fan ₹30,278,407; Aurora Kettle ₹24,091,861; Flux Mixer Grinder ₹22,321,476; Glow LED Lamp ₹12,884,916; Halo Smart Bulb ₹5,684,360; Ember Room Heater ₹2,909,900. Top: Cascade Water Purifier.</t>
+          <t>Proposal table, then line chart with all regions summed: April 1,095; May 1,469; June 1,150; July 598; August 398; September 323.</t>
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>Exact values (page-computed).</t>
+          <t>Values match exactly; source shows Sales_FY27_H1.xlsx sheet Transactions.</t>
         </is>
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>2 = exact; 0 = otherwise.</t>
+          <t>2 = exact values and plotted after confirm; 1 = right shape, wrong grouping; 0 = wrong numbers.</t>
         </is>
       </c>
       <c r="H14" s="12" t="inlineStr">
@@ -1664,7 +1664,7 @@
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>B5</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -1679,17 +1679,17 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Show net revenue by region as a bar chart.</t>
+          <t>Bar chart of total net revenue by product for H1.</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Values (₹): West ₹50,698,392; North ₹48,128,931; South ₹43,368,264; East ₹35,413,779.</t>
+          <t>Bar chart, values (₹): Cascade Water Purifier ₹40,085,016; Drift Air Cooler ₹39,353,430; Breeze Fan ₹30,278,407; Aurora Kettle ₹24,091,861; Flux Mixer Grinder ₹22,321,476; Glow LED Lamp ₹12,884,916; Halo Smart Bulb ₹5,684,360; Ember Room Heater ₹2,909,900. Top: Cascade Water Purifier.</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>Exact values.</t>
+          <t>Exact values (page-computed).</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
@@ -1712,7 +1712,7 @@
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>B6</t>
+          <t>B5</t>
         </is>
       </c>
       <c r="B16" s="12" t="inlineStr">
@@ -1722,32 +1722,32 @@
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>Aggregate (text answer)</t>
+          <t>Chart (exact numbers)</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>Which product earned the most net revenue in H1, and how much?</t>
+          <t>Show net revenue by region as a bar chart.</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Cascade Water Purifier, ₹40,085,016 (₹400.9 lakh).</t>
+          <t>Values (₹): West ₹50,698,392; North ₹48,128,931; South ₹43,368,264; East ₹35,413,779.</t>
         </is>
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>Product name and amount within 1%.</t>
+          <t>Exact values.</t>
         </is>
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>2 = right product and amount; 1 = right product, wrong/missing amount, or says it can only see part of the data; 0 = wrong product stated confidently.</t>
+          <t>2 = exact; 0 = otherwise.</t>
         </is>
       </c>
       <c r="H16" s="12" t="inlineStr">
         <is>
-          <t>Default settings; check the 'Exact figures calculated by the page' table under the answer</t>
+          <t>Default settings</t>
         </is>
       </c>
       <c r="I16" s="13" t="n"/>
@@ -1760,7 +1760,7 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>B7</t>
+          <t>B6</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -1775,27 +1775,27 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>What was total net revenue for H1 across all products and regions?</t>
+          <t>Which product earned the most net revenue in H1, and how much?</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>₹177,609,366 (₹1,776.1 lakh).</t>
+          <t>Cascade Water Purifier, ₹40,085,016 (₹400.9 lakh).</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Within 1%, or an honest statement that the full total can't be computed from the passages it sees.</t>
+          <t>Product name and amount within 1%.</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>2 = correct; 1 = honest 'can't compute all rows'; 0 = a wrong number stated as fact.</t>
+          <t>2 = right product and amount; 1 = right product, wrong/missing amount, or says it can only see part of the data; 0 = wrong product stated confidently.</t>
         </is>
       </c>
       <c r="H17" s="12" t="inlineStr">
         <is>
-          <t>Default settings; check the calculated table under the answer</t>
+          <t>Default settings; check the 'Exact figures calculated by the page' table under the answer</t>
         </is>
       </c>
       <c r="I17" s="13" t="n"/>
@@ -1808,7 +1808,7 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>B8</t>
+          <t>B7</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
@@ -1823,22 +1823,22 @@
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Which products missed their H1 unit target?</t>
+          <t>What was total net revenue for H1 across all products and regions?</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Missed: Cascade Water Purifier (3,246 vs target 3,700), Ember Room Heater (1,145 vs target 1,400), Flux Mixer Grinder (5,109 vs target 5,400), Halo Smart Bulb (4,890 vs target 6,400).</t>
+          <t>₹177,609,366 (₹1,776.1 lakh).</t>
         </is>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Exactly these products.</t>
+          <t>Within 1%, or an honest statement that the full total can't be computed from the passages it sees.</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>2 = exact list; 1 = partial or honest limitation; 0 = wrong list stated as fact.</t>
+          <t>2 = correct; 1 = honest 'can't compute all rows'; 0 = a wrong number stated as fact.</t>
         </is>
       </c>
       <c r="H18" s="12" t="inlineStr">
@@ -1856,7 +1856,7 @@
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>B9</t>
+          <t>B8</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -1866,32 +1866,32 @@
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>Summary</t>
+          <t>Aggregate (text answer)</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Summarise how the Halo Smart Bulb has done since launch.</t>
+          <t>Which products missed their H1 unit target?</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Launched June 2026 with a 15% introductory discount; units grew every month (June 501; July 1,078; August 1,513; September 1,798); app pairing problems reported by customers and stores; app fix in progress.</t>
+          <t>Missed: Cascade Water Purifier (3,246 vs target 3,700), Ember Room Heater (1,145 vs target 1,400), Flux Mixer Grinder (5,109 vs target 5,400), Halo Smart Bulb (4,890 vs target 6,400).</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>Launch month, discount, growth, pairing issue.</t>
+          <t>Exactly these products.</t>
         </is>
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>2 = all four; 1 = two or three; 0 = otherwise.</t>
+          <t>2 = exact list; 1 = partial or honest limitation; 0 = wrong list stated as fact.</t>
         </is>
       </c>
       <c r="H19" s="12" t="inlineStr">
         <is>
-          <t>Default settings</t>
+          <t>Default settings; check the calculated table under the answer</t>
         </is>
       </c>
       <c r="I19" s="13" t="n"/>
@@ -1904,7 +1904,7 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>B10</t>
+          <t>B9</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
@@ -1914,27 +1914,27 @@
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>Negative (not in documents)</t>
+          <t>Summary</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>What were sales in October 2026?</t>
+          <t>Summarise how the Halo Smart Bulb has done since launch.</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Not in the data (the data covers April to September 2026). Should say it couldn't find this.</t>
+          <t>Launched June 2026 with a 15% introductory discount; units grew every month (June 501; July 1,078; August 1,513; September 1,798); app pairing problems reported by customers and stores; app fix in progress.</t>
         </is>
       </c>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>Must not invent October figures.</t>
+          <t>Launch month, discount, growth, pairing issue.</t>
         </is>
       </c>
       <c r="G20" s="12" t="inlineStr">
         <is>
-          <t>2 = says not found / data ends September; 0 = any invented figure.</t>
+          <t>2 = all four; 1 = two or three; 0 = otherwise.</t>
         </is>
       </c>
       <c r="H20" s="12" t="inlineStr">
@@ -1949,13 +1949,61 @@
       <c r="M20" s="13" t="n"/>
       <c r="N20" s="13" t="n"/>
     </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>B10</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>B: Sales</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Negative (not in documents)</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>What were sales in October 2026?</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>Not in the data (the data covers April to September 2026). Should say it couldn't find this.</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>Must not invent October figures.</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="inlineStr">
+        <is>
+          <t>2 = says not found / data ends September; 0 = any invented figure.</t>
+        </is>
+      </c>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>Default settings</t>
+        </is>
+      </c>
+      <c r="I21" s="13" t="n"/>
+      <c r="J21" s="13" t="n"/>
+      <c r="K21" s="13" t="n"/>
+      <c r="L21" s="13" t="n"/>
+      <c r="M21" s="13" t="n"/>
+      <c r="N21" s="13" t="n"/>
+    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="J3:J20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
+    <dataValidation sqref="J3:J21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>2</formula2>
     </dataValidation>
-    <dataValidation sqref="K3:L20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K3:L21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Check every document before answering "not found"
Claude now always receives the list of all documents and is told to go
through each one, judging whether it contains the answer or lets it be
worked out, before saying no. A "no" must come through the new
report_not_found tool with one reason per document, shown under the
answer as a "How I checked" table. The page no longer answers
"not found" on its own when no passage matches; every question reaches
Claude. The A8 reference answer now expects the per-document check.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/local-qa/eval/Evaluation_Scoresheet.xlsx
+++ b/local-qa/eval/Evaluation_Scoresheet.xlsx
@@ -1444,17 +1444,17 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Not in the documents. The tool should answer that it couldn't find this.</t>
+          <t>Not in the documents. The tool should say it couldn't find this, with a 'How I checked' table giving each of the documents and why it can't answer.</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>Must not invent anything.</t>
+          <t>Must not invent anything; every document checked.</t>
         </is>
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>2 = says not found; 0 = any invented content.</t>
+          <t>2 = not found with a check per document; 1 = not found without the checks; 0 = any invented content.</t>
         </is>
       </c>
       <c r="H10" s="12" t="inlineStr">

</xml_diff>